<commit_message>
data: actualizar pipeline Excel
</commit_message>
<xml_diff>
--- a/data/PIPE LINE PROCESO COMERCIAL - Ventas TA.xlsx
+++ b/data/PIPE LINE PROCESO COMERCIAL - Ventas TA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlando.carvajal.DESMEX\Desktop\ClaudeCode\Pipeline1\pipeline-web\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06111943-CD1E-4FE6-9C9F-BA263163C4F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{46E7B812-D90F-416E-B00A-14D1BCEEBAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
     <sheet name="Copia seguridad 27-01-2026" sheetId="9" state="hidden" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Alexandro Carrasco'!$A$1:$L$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Alexandro Carrasco'!$A$1:$L$214</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Copia seguridad 27-01-2026'!$A$1:$K$275</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Daniela Lara'!$A$1:$L$115</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Josué Morales'!$A$1:$K$148</definedName>
@@ -50,11 +50,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={e486e15b-6e62-4266-9919-8644122bfe6b}</author>
-    <author>tc={c7ed0c02-4231-43e4-b355-89166dd53e3e}</author>
+    <author>tc={b3541e79-7142-4e55-b220-7706f78da251}</author>
+    <author>tc={fd5a665c-4ee9-467e-b1ab-105dbaf1c13e}</author>
   </authors>
   <commentList>
-    <comment ref="J32" authorId="0" shapeId="0" xr:uid="{E486E15B-6E62-4266-9919-8644122BFE6B}">
+    <comment ref="J32" authorId="0" shapeId="0" xr:uid="{B3541E79-7142-4E55-B220-7706F78DA251}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,7 +62,7 @@
     ya lo tiene en seguimiento Josué</t>
       </text>
     </comment>
-    <comment ref="J62" authorId="1" shapeId="0" xr:uid="{C7ED0C02-4231-43E4-B355-89166DD53E3E}">
+    <comment ref="J62" authorId="1" shapeId="0" xr:uid="{FD5A665C-4EE9-467E-B1AB-105DBAF1C13E}">
       <text>
         <t>[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4782" uniqueCount="1467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4784" uniqueCount="1468">
   <si>
     <t>ID de Prospecto</t>
   </si>
@@ -3759,6 +3759,9 @@
   </si>
   <si>
     <t>Polesazinc</t>
+  </si>
+  <si>
+    <t>Arq. Alejandra Vergara</t>
   </si>
   <si>
     <r>
@@ -5757,7 +5760,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Anónimo" id="{55861A80-B128-4B50-9A2A-1BD4FD1E5499}" userId="" providerId="google-sheets"/>
+  <person displayName="Anónimo" id="{800B8EA1-66A5-4344-9FAA-9DC8A887D0FD}" userId="" providerId="google-sheets"/>
 </personList>
 </file>
 
@@ -5803,7 +5806,17 @@
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabla_6" displayName="Tabla_6" ref="A1:L115">
-  <autoFilter ref="A1:L115" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+  <autoFilter ref="A1:L115" xr:uid="{00000000-0009-0000-0100-000004000000}">
+    <filterColumn colId="5">
+      <filters blank="1">
+        <filter val="10. Negociación"/>
+        <filter val="5. Visita Técnica / Diagnóstico en Sitio"/>
+        <filter val="6. Diseño de Solución / Pre-Ingeniería"/>
+        <filter val="7. Estimación / Cotización"/>
+        <filter val="8. Propuesta Enviada"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="ID de Prospecto"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Nombre del Prospecto"/>
@@ -5823,8 +5836,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabla_3" displayName="Tabla_3" ref="A1:L213">
-  <autoFilter ref="A1:L213" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Tabla_3" displayName="Tabla_3" ref="A1:L214">
+  <autoFilter ref="A1:L214" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="ID de Prospecto"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Nombre del Prospecto"/>
@@ -6101,10 +6114,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="J32" dT="2026-02-23T14:39:40.00" personId="{55861A80-B128-4B50-9A2A-1BD4FD1E5499}" id="{E486E15B-6E62-4266-9919-8644122BFE6B}" done="1">
+  <threadedComment ref="J32" dT="2026-02-23T14:39:40.00" personId="{800B8EA1-66A5-4344-9FAA-9DC8A887D0FD}" id="{B3541E79-7142-4E55-B220-7706F78DA251}" done="1">
     <text>ya lo tiene en seguimiento Josué</text>
   </threadedComment>
-  <threadedComment ref="J62" dT="2026-02-24T22:06:20.00" personId="{55861A80-B128-4B50-9A2A-1BD4FD1E5499}" id="{C7ED0C02-4231-43E4-B355-89166DD53E3E}" done="1">
+  <threadedComment ref="J62" dT="2026-02-24T22:06:20.00" personId="{800B8EA1-66A5-4344-9FAA-9DC8A887D0FD}" id="{FD5A665C-4EE9-467E-B1AB-105DBAF1C13E}" done="1">
     <text>Ya tienen contrato con Ammper</text>
   </threadedComment>
 </ThreadedComments>
@@ -11939,7 +11952,7 @@
       <c r="AB1" s="7"/>
       <c r="AC1" s="7"/>
     </row>
-    <row r="2" spans="1:29" ht="22.5" customHeight="1">
+    <row r="2" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A2" s="46" t="s">
         <v>445</v>
       </c>
@@ -11975,7 +11988,7 @@
       </c>
       <c r="L2" s="57"/>
     </row>
-    <row r="3" spans="1:29" ht="22.5" customHeight="1">
+    <row r="3" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A3" s="46" t="s">
         <v>451</v>
       </c>
@@ -12011,7 +12024,7 @@
       </c>
       <c r="L3" s="57"/>
     </row>
-    <row r="4" spans="1:29" ht="22.5" customHeight="1">
+    <row r="4" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A4" s="46" t="s">
         <v>454</v>
       </c>
@@ -12047,7 +12060,7 @@
       </c>
       <c r="L4" s="57"/>
     </row>
-    <row r="5" spans="1:29" ht="22.5" customHeight="1">
+    <row r="5" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A5" s="46" t="s">
         <v>457</v>
       </c>
@@ -12083,7 +12096,7 @@
       </c>
       <c r="L5" s="57"/>
     </row>
-    <row r="6" spans="1:29" ht="22.5" customHeight="1">
+    <row r="6" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A6" s="46" t="s">
         <v>668</v>
       </c>
@@ -12119,7 +12132,7 @@
       </c>
       <c r="L6" s="57"/>
     </row>
-    <row r="7" spans="1:29" ht="22.5" customHeight="1">
+    <row r="7" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A7" s="46" t="s">
         <v>459</v>
       </c>
@@ -12191,7 +12204,7 @@
       </c>
       <c r="L8" s="57"/>
     </row>
-    <row r="9" spans="1:29" ht="22.5" customHeight="1">
+    <row r="9" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A9" s="46" t="s">
         <v>465</v>
       </c>
@@ -12227,7 +12240,7 @@
       </c>
       <c r="L9" s="57"/>
     </row>
-    <row r="10" spans="1:29" ht="22.5" customHeight="1">
+    <row r="10" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A10" s="46" t="s">
         <v>468</v>
       </c>
@@ -12263,7 +12276,7 @@
       </c>
       <c r="L10" s="57"/>
     </row>
-    <row r="11" spans="1:29" ht="22.5" customHeight="1">
+    <row r="11" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A11" s="46" t="s">
         <v>471</v>
       </c>
@@ -12299,7 +12312,7 @@
       </c>
       <c r="L11" s="57"/>
     </row>
-    <row r="12" spans="1:29" ht="22.5" customHeight="1">
+    <row r="12" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A12" s="46" t="s">
         <v>474</v>
       </c>
@@ -12335,7 +12348,7 @@
       </c>
       <c r="L12" s="57"/>
     </row>
-    <row r="13" spans="1:29" ht="22.5" customHeight="1">
+    <row r="13" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A13" s="46" t="s">
         <v>477</v>
       </c>
@@ -12371,7 +12384,7 @@
       </c>
       <c r="L13" s="57"/>
     </row>
-    <row r="14" spans="1:29" ht="22.5" customHeight="1">
+    <row r="14" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A14" s="46" t="s">
         <v>481</v>
       </c>
@@ -12443,7 +12456,7 @@
       </c>
       <c r="L15" s="57"/>
     </row>
-    <row r="16" spans="1:29" ht="22.5" customHeight="1">
+    <row r="16" spans="1:29" ht="22.5" hidden="1" customHeight="1">
       <c r="A16" s="46" t="s">
         <v>488</v>
       </c>
@@ -12587,7 +12600,7 @@
       </c>
       <c r="L19" s="57"/>
     </row>
-    <row r="20" spans="1:12" ht="22.5" customHeight="1">
+    <row r="20" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A20" s="46" t="s">
         <v>500</v>
       </c>
@@ -12659,7 +12672,7 @@
       </c>
       <c r="L21" s="57"/>
     </row>
-    <row r="22" spans="1:12" ht="22.5" customHeight="1">
+    <row r="22" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A22" s="46" t="s">
         <v>506</v>
       </c>
@@ -12695,7 +12708,7 @@
       </c>
       <c r="L22" s="57"/>
     </row>
-    <row r="23" spans="1:12" ht="22.5" customHeight="1">
+    <row r="23" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A23" s="46" t="s">
         <v>510</v>
       </c>
@@ -12767,7 +12780,7 @@
       </c>
       <c r="L24" s="57"/>
     </row>
-    <row r="25" spans="1:12" ht="22.5" customHeight="1">
+    <row r="25" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A25" s="46" t="s">
         <v>517</v>
       </c>
@@ -12803,7 +12816,7 @@
       </c>
       <c r="L25" s="57"/>
     </row>
-    <row r="26" spans="1:12" ht="22.5" customHeight="1">
+    <row r="26" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A26" s="46" t="s">
         <v>520</v>
       </c>
@@ -12837,7 +12850,7 @@
       </c>
       <c r="L26" s="57"/>
     </row>
-    <row r="27" spans="1:12" ht="22.5" customHeight="1">
+    <row r="27" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A27" s="46" t="s">
         <v>523</v>
       </c>
@@ -12873,7 +12886,7 @@
       </c>
       <c r="L27" s="57"/>
     </row>
-    <row r="28" spans="1:12" ht="22.5" customHeight="1">
+    <row r="28" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A28" s="46" t="s">
         <v>527</v>
       </c>
@@ -12909,7 +12922,7 @@
       </c>
       <c r="L28" s="57"/>
     </row>
-    <row r="29" spans="1:12" ht="22.5" customHeight="1">
+    <row r="29" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A29" s="46" t="s">
         <v>531</v>
       </c>
@@ -12945,7 +12958,7 @@
       </c>
       <c r="L29" s="57"/>
     </row>
-    <row r="30" spans="1:12" ht="22.5" customHeight="1">
+    <row r="30" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A30" s="46" t="s">
         <v>534</v>
       </c>
@@ -12981,7 +12994,7 @@
       </c>
       <c r="L30" s="57"/>
     </row>
-    <row r="31" spans="1:12" ht="22.5" customHeight="1">
+    <row r="31" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A31" s="46" t="s">
         <v>538</v>
       </c>
@@ -13017,7 +13030,7 @@
       </c>
       <c r="L31" s="57"/>
     </row>
-    <row r="32" spans="1:12" ht="22.5" customHeight="1">
+    <row r="32" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A32" s="46" t="s">
         <v>541</v>
       </c>
@@ -13089,7 +13102,7 @@
       </c>
       <c r="L33" s="57"/>
     </row>
-    <row r="34" spans="1:12" ht="22.5" customHeight="1">
+    <row r="34" spans="1:12" ht="22.5" hidden="1" customHeight="1">
       <c r="A34" s="46" t="s">
         <v>547</v>
       </c>
@@ -14668,7 +14681,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC213"/>
+  <dimension ref="A1:AC214"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.609375" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="17.21875" customWidth="1"/>
@@ -14754,7 +14767,7 @@
         <v>448</v>
       </c>
       <c r="F2" s="53" t="s">
-        <v>24</v>
+        <v>102</v>
       </c>
       <c r="G2" s="54">
         <v>46111</v>
@@ -21331,21 +21344,39 @@
       <c r="K213" s="46"/>
       <c r="L213" s="46"/>
     </row>
+    <row r="214" spans="1:12" ht="22.5" customHeight="1">
+      <c r="A214" s="46"/>
+      <c r="B214" s="9" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C214" s="46"/>
+      <c r="D214" s="10"/>
+      <c r="E214" s="10" t="s">
+        <v>448</v>
+      </c>
+      <c r="F214" s="53"/>
+      <c r="G214" s="54"/>
+      <c r="H214" s="55"/>
+      <c r="I214" s="56"/>
+      <c r="J214" s="53"/>
+      <c r="K214" s="46"/>
+      <c r="L214" s="46"/>
+    </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" sqref="F2:F213" xr:uid="{00000000-0002-0000-0400-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F214" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"1. Prospección,2. Contacto Inicial,3. Calificación,4. Levantamiento de Requerimientos,5. Visita Técnica / Diagnóstico en Sitio,6. Diseño de Solución / Pre-Ingeniería,7. Estimación / Cotización,8. Propuesta Enviada,9. Aclaraciones / Ajustes de Propuesta,10"&amp;". Negociación,11. Aprobación Interna (Go/No-Go),12. Cierre de Venta (Contrato / OC),13. Kickoff / Inicio de Proyecto,14. Descartado / No Califica,15. En Pausa / Seguimiento Posterior"</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="G2:G213" xr:uid="{00000000-0002-0000-0400-000001000000}">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="G2:G214" xr:uid="{00000000-0002-0000-0400-000001000000}">
       <formula1>OR(NOT(ISERROR(DATEVALUE(G2))), AND(ISNUMBER(G2), LEFT(CELL("format", G2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="H2:I213" xr:uid="{00000000-0002-0000-0400-000002000000}">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="H2:I214" xr:uid="{00000000-0002-0000-0400-000002000000}">
       <formula1>AND(ISNUMBER(H2),(NOT(OR(NOT(ISERROR(DATEVALUE(H2))), AND(ISNUMBER(H2), LEFT(CELL("format", H2))="D")))))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J2:J213" xr:uid="{00000000-0002-0000-0400-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J214" xr:uid="{00000000-0002-0000-0400-000003000000}">
       <formula1>"Referido (Cliente),Referido (Proveedor/Subcontratista),Referido (Empleado/Interno),Cliente Recurrente (Recompra/Ampliación),Sitio Web (Formulario),Landing Page (Campaña),Chat Web / WhatsApp,SEO (Búsqueda Orgánica),Google Ads (Search),Remarketing (Display/"&amp;"Redes),LinkedIn (Orgánico),Email Outbound (Prospección),Llamada en Frío (Prospección),Visita en Frío (Prospección),Feria / Expo Industrial,Congreso / Cámara / Networking,Webinar / Evento Virtual,Licitación Pública,Licitación Privada (RFP/RFQ),Portal de Co"&amp;"mpras (Cliente),Alianza (Integrador/EPC/Constructor),Partner Tecnológico (Marca/Distribuidor),Directorio B2B / Clúster,Redes Sociales (Facebook/Instagram),YouTube / Contenido Técnico,PR / Medio Especializado,Reactivación de Base de Datos,Otros"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="B2:C213 E2:E213 K2:K213" xr:uid="{00000000-0002-0000-0400-000004000000}"/>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="B2:C214 E2:E214 K2:K214" xr:uid="{00000000-0002-0000-0400-000004000000}"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
@@ -21611,10 +21642,10 @@
         <v>481</v>
       </c>
       <c r="B2" s="69" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="D2" s="70"/>
       <c r="E2" s="70"/>
@@ -21634,7 +21665,7 @@
         <v>25</v>
       </c>
       <c r="K2" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="21" customHeight="1">
@@ -21642,10 +21673,10 @@
         <v>484</v>
       </c>
       <c r="B3" s="77" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="C3" s="76" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="D3" s="70"/>
       <c r="E3" s="70"/>
@@ -21663,7 +21694,7 @@
         <v>74</v>
       </c>
       <c r="K3" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="22.5" customHeight="1">
@@ -21671,10 +21702,10 @@
         <v>488</v>
       </c>
       <c r="B4" s="81" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="D4" s="83"/>
       <c r="E4" s="70"/>
@@ -21692,7 +21723,7 @@
         <v>25</v>
       </c>
       <c r="K4" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="22.5" customHeight="1">
@@ -21700,10 +21731,10 @@
         <v>491</v>
       </c>
       <c r="B5" s="81" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="C5" s="82" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="D5" s="83"/>
       <c r="E5" s="70"/>
@@ -21721,7 +21752,7 @@
         <v>782</v>
       </c>
       <c r="K5" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="22.5" customHeight="1">
@@ -21729,10 +21760,10 @@
         <v>494</v>
       </c>
       <c r="B6" s="81" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="C6" s="82" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="D6" s="83"/>
       <c r="E6" s="70"/>
@@ -21750,7 +21781,7 @@
         <v>74</v>
       </c>
       <c r="K6" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="22.5" customHeight="1">
@@ -21758,10 +21789,10 @@
         <v>497</v>
       </c>
       <c r="B7" s="77" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="C7" s="76" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="D7" s="70"/>
       <c r="E7" s="70"/>
@@ -21777,7 +21808,7 @@
         <v>25</v>
       </c>
       <c r="K7" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="22.5" customHeight="1">
@@ -21785,10 +21816,10 @@
         <v>500</v>
       </c>
       <c r="B8" s="77" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="C8" s="76" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="D8" s="70"/>
       <c r="E8" s="70"/>
@@ -21806,7 +21837,7 @@
         <v>74</v>
       </c>
       <c r="K8" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="22.5" customHeight="1">
@@ -21814,10 +21845,10 @@
         <v>503</v>
       </c>
       <c r="B9" s="81" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="C9" s="82" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="D9" s="83"/>
       <c r="E9" s="70"/>
@@ -21835,7 +21866,7 @@
         <v>74</v>
       </c>
       <c r="K9" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="22.5" customHeight="1">
@@ -21843,10 +21874,10 @@
         <v>506</v>
       </c>
       <c r="B10" s="76" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="C10" s="76" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="D10" s="70"/>
       <c r="E10" s="70"/>
@@ -21864,7 +21895,7 @@
         <v>25</v>
       </c>
       <c r="K10" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="22.5" customHeight="1">
@@ -21872,10 +21903,10 @@
         <v>514</v>
       </c>
       <c r="B11" s="81" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C11" s="82" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="D11" s="83"/>
       <c r="E11" s="70"/>
@@ -21893,7 +21924,7 @@
         <v>74</v>
       </c>
       <c r="K11" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="22.5" customHeight="1">
@@ -21901,10 +21932,10 @@
         <v>517</v>
       </c>
       <c r="B12" s="81" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="C12" s="82" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="D12" s="83"/>
       <c r="E12" s="70"/>
@@ -21922,7 +21953,7 @@
         <v>74</v>
       </c>
       <c r="K12" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="22.5" customHeight="1">
@@ -21930,10 +21961,10 @@
         <v>520</v>
       </c>
       <c r="B13" s="77" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="C13" s="76" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="D13" s="70"/>
       <c r="E13" s="70"/>
@@ -21951,7 +21982,7 @@
         <v>25</v>
       </c>
       <c r="K13" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="22.5" customHeight="1">
@@ -21959,10 +21990,10 @@
         <v>523</v>
       </c>
       <c r="B14" s="81" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="C14" s="82" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="D14" s="83"/>
       <c r="E14" s="70"/>
@@ -21978,7 +22009,7 @@
         <v>74</v>
       </c>
       <c r="K14" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="22.5" customHeight="1">
@@ -21986,10 +22017,10 @@
         <v>527</v>
       </c>
       <c r="B15" s="99" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="C15" s="82" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D15" s="83"/>
       <c r="E15" s="70"/>
@@ -22007,7 +22038,7 @@
         <v>74</v>
       </c>
       <c r="K15" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="22.5" customHeight="1">
@@ -22015,10 +22046,10 @@
         <v>531</v>
       </c>
       <c r="B16" s="77" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="D16" s="70"/>
       <c r="E16" s="70"/>
@@ -22034,7 +22065,7 @@
         <v>25</v>
       </c>
       <c r="K16" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="22.5" customHeight="1">
@@ -22042,10 +22073,10 @@
         <v>534</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="D17" s="70"/>
       <c r="E17" s="70"/>
@@ -22065,7 +22096,7 @@
         <v>25</v>
       </c>
       <c r="K17" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="22.5" customHeight="1">
@@ -22073,10 +22104,10 @@
         <v>538</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="70"/>
@@ -22096,7 +22127,7 @@
         <v>74</v>
       </c>
       <c r="K18" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="22.5" customHeight="1">
@@ -22104,10 +22135,10 @@
         <v>541</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="11"/>
@@ -22127,7 +22158,7 @@
         <v>513</v>
       </c>
       <c r="K19" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="22.5" customHeight="1">
@@ -22135,10 +22166,10 @@
         <v>544</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="C20" s="76" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
@@ -22156,7 +22187,7 @@
         <v>25</v>
       </c>
       <c r="K20" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="22.5" customHeight="1">
@@ -22164,10 +22195,10 @@
         <v>547</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="C21" s="76" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
@@ -22185,7 +22216,7 @@
         <v>745</v>
       </c>
       <c r="K21" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="22.5" customHeight="1">
@@ -22193,10 +22224,10 @@
         <v>552</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="C22" s="76" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="D22" s="10"/>
       <c r="E22" s="11"/>
@@ -22214,7 +22245,7 @@
         <v>551</v>
       </c>
       <c r="K22" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="22.5" customHeight="1">
@@ -22222,10 +22253,10 @@
         <v>555</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="C23" s="76" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="D23" s="10"/>
       <c r="E23" s="11"/>
@@ -22243,7 +22274,7 @@
         <v>551</v>
       </c>
       <c r="K23" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="22.5" customHeight="1">
@@ -22251,10 +22282,10 @@
         <v>558</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C24" s="76" t="s">
         <v>1271</v>
-      </c>
-      <c r="C24" s="76" t="s">
-        <v>1270</v>
       </c>
       <c r="D24" s="10"/>
       <c r="E24" s="11"/>
@@ -22272,7 +22303,7 @@
         <v>551</v>
       </c>
       <c r="K24" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="22.5" customHeight="1">
@@ -22280,10 +22311,10 @@
         <v>558</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="D25" s="10"/>
       <c r="E25" s="11"/>
@@ -22303,7 +22334,7 @@
         <v>513</v>
       </c>
       <c r="K25" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="22.5" customHeight="1">
@@ -22311,10 +22342,10 @@
         <v>558</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="D26" s="10"/>
       <c r="E26" s="11"/>
@@ -22334,7 +22365,7 @@
         <v>551</v>
       </c>
       <c r="K26" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="22.5" customHeight="1">
@@ -22342,10 +22373,10 @@
         <v>562</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="D27" s="10"/>
       <c r="E27" s="11"/>
@@ -22363,7 +22394,7 @@
         <v>513</v>
       </c>
       <c r="K27" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="22.5" customHeight="1">
@@ -22371,10 +22402,10 @@
         <v>565</v>
       </c>
       <c r="B28" s="9" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>1278</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>1277</v>
       </c>
       <c r="D28" s="10"/>
       <c r="E28" s="11"/>
@@ -22392,7 +22423,7 @@
         <v>513</v>
       </c>
       <c r="K28" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="22.5" customHeight="1">
@@ -22400,10 +22431,10 @@
         <v>568</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="D29" s="10"/>
       <c r="E29" s="11"/>
@@ -22419,7 +22450,7 @@
       <c r="I29" s="45"/>
       <c r="J29" s="14"/>
       <c r="K29" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
   </sheetData>
@@ -22542,10 +22573,10 @@
         <v>445</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="D2" s="101"/>
       <c r="E2" s="101" t="s">
@@ -22563,7 +22594,7 @@
         <v>782</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="22.5" customHeight="1">
@@ -22571,10 +22602,10 @@
         <v>451</v>
       </c>
       <c r="B3" s="46" t="s">
-        <v>1284</v>
+        <v>1285</v>
       </c>
       <c r="C3" s="46" t="s">
-        <v>1285</v>
+        <v>1286</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10" t="s">
@@ -22596,7 +22627,7 @@
         <v>782</v>
       </c>
       <c r="K3" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="22.5" customHeight="1">
@@ -22604,14 +22635,14 @@
         <v>454</v>
       </c>
       <c r="B4" s="51" t="s">
-        <v>1286</v>
+        <v>1287</v>
       </c>
       <c r="C4" s="46" t="s">
-        <v>1287</v>
+        <v>1288</v>
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="10" t="s">
-        <v>1288</v>
+        <v>1289</v>
       </c>
       <c r="F4" s="53" t="s">
         <v>449</v>
@@ -22625,7 +22656,7 @@
         <v>782</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="22.5" customHeight="1">
@@ -22633,10 +22664,10 @@
         <v>457</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>1289</v>
+        <v>1290</v>
       </c>
       <c r="C5" s="46" t="s">
-        <v>1290</v>
+        <v>1291</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="10" t="s">
@@ -22658,7 +22689,7 @@
         <v>688</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="22.5" customHeight="1">
@@ -22666,10 +22697,10 @@
         <v>668</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>1291</v>
+        <v>1292</v>
       </c>
       <c r="C6" s="46" t="s">
-        <v>1292</v>
+        <v>1293</v>
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="10" t="s">
@@ -22687,7 +22718,7 @@
         <v>688</v>
       </c>
       <c r="K6" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="7" spans="1:29" ht="22.5" customHeight="1">
@@ -22695,10 +22726,10 @@
         <v>459</v>
       </c>
       <c r="B7" s="51" t="s">
-        <v>1293</v>
+        <v>1294</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>1294</v>
+        <v>1295</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10" t="s">
@@ -22716,7 +22747,7 @@
         <v>782</v>
       </c>
       <c r="K7" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="22.5" customHeight="1">
@@ -22724,10 +22755,10 @@
         <v>462</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>1295</v>
+        <v>1296</v>
       </c>
       <c r="C8" s="46" t="s">
-        <v>1296</v>
+        <v>1297</v>
       </c>
       <c r="D8" s="10"/>
       <c r="E8" s="10" t="s">
@@ -22745,7 +22776,7 @@
         <v>25</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="22.5" customHeight="1">
@@ -22753,14 +22784,14 @@
         <v>465</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>1297</v>
+        <v>1298</v>
       </c>
       <c r="C9" s="46" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="F9" s="53" t="s">
         <v>40</v>
@@ -22774,7 +22805,7 @@
         <v>659</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="22.5" customHeight="1">
@@ -22782,10 +22813,10 @@
         <v>468</v>
       </c>
       <c r="B10" s="51" t="s">
-        <v>1300</v>
+        <v>1301</v>
       </c>
       <c r="C10" s="46" t="s">
-        <v>1301</v>
+        <v>1302</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10" t="s">
@@ -22803,7 +22834,7 @@
         <v>659</v>
       </c>
       <c r="K10" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="22.5" customHeight="1">
@@ -22811,14 +22842,14 @@
         <v>471</v>
       </c>
       <c r="B11" s="51" t="s">
-        <v>1302</v>
+        <v>1303</v>
       </c>
       <c r="C11" s="46" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10" t="s">
-        <v>1299</v>
+        <v>1300</v>
       </c>
       <c r="F11" s="53" t="s">
         <v>32</v>
@@ -22832,7 +22863,7 @@
         <v>659</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="22.5" customHeight="1">
@@ -22840,10 +22871,10 @@
         <v>474</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
       <c r="C12" s="46" t="s">
-        <v>1305</v>
+        <v>1306</v>
       </c>
       <c r="D12" s="10"/>
       <c r="E12" s="10" t="s">
@@ -22859,7 +22890,7 @@
         <v>659</v>
       </c>
       <c r="K12" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="13" spans="1:29" ht="22.5" customHeight="1">
@@ -22867,10 +22898,10 @@
         <v>477</v>
       </c>
       <c r="B13" s="51" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>1307</v>
+        <v>1308</v>
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10" t="s">
@@ -22892,7 +22923,7 @@
         <v>659</v>
       </c>
       <c r="K13" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="22.5" customHeight="1">
@@ -22900,10 +22931,10 @@
         <v>481</v>
       </c>
       <c r="B14" s="51" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="C14" s="51" t="s">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="D14" s="10"/>
       <c r="E14" s="10" t="s">
@@ -22923,7 +22954,7 @@
         <v>782</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="22.5" customHeight="1">
@@ -22931,10 +22962,10 @@
         <v>484</v>
       </c>
       <c r="B15" s="51" t="s">
-        <v>1309</v>
+        <v>1310</v>
       </c>
       <c r="C15" s="51" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10" t="s">
@@ -22954,10 +22985,10 @@
         <v>488</v>
       </c>
       <c r="B16" s="51" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="C16" s="51" t="s">
-        <v>1312</v>
+        <v>1313</v>
       </c>
       <c r="D16" s="10"/>
       <c r="E16" s="10" t="s">
@@ -22977,7 +23008,7 @@
         <v>659</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="22.5" customHeight="1">
@@ -22985,10 +23016,10 @@
         <v>491</v>
       </c>
       <c r="B17" s="51" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="C17" s="51" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10" t="s">
@@ -23008,10 +23039,10 @@
         <v>494</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>1313</v>
+        <v>1314</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="D18" s="10"/>
       <c r="E18" s="10" t="s">
@@ -23031,10 +23062,10 @@
         <v>497</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>1317</v>
+        <v>1318</v>
       </c>
       <c r="D19" s="10"/>
       <c r="E19" s="10" t="s">
@@ -23054,10 +23085,10 @@
         <v>500</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>1318</v>
+        <v>1319</v>
       </c>
       <c r="C20" s="51" t="s">
-        <v>1319</v>
+        <v>1320</v>
       </c>
       <c r="D20" s="10"/>
       <c r="E20" s="10" t="s">
@@ -23217,7 +23248,7 @@
         <v>782</v>
       </c>
       <c r="K2" s="104" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="22.5" customHeight="1">
@@ -23225,10 +23256,10 @@
         <v>471</v>
       </c>
       <c r="B3" s="81" t="s">
-        <v>1321</v>
+        <v>1322</v>
       </c>
       <c r="C3" s="82" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="D3" s="83"/>
       <c r="E3" s="83"/>
@@ -23244,7 +23275,7 @@
         <v>74</v>
       </c>
       <c r="K3" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="22.5" customHeight="1">
@@ -23532,10 +23563,10 @@
         <v>474</v>
       </c>
       <c r="B14" s="107" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="C14" s="108" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="D14" s="109"/>
       <c r="E14" s="109"/>
@@ -23553,7 +23584,7 @@
         <v>74</v>
       </c>
       <c r="K14" s="115" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="22.5" customHeight="1">
@@ -23843,10 +23874,10 @@
         <v>477</v>
       </c>
       <c r="B25" s="117" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="C25" s="118" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="D25" s="119"/>
       <c r="E25" s="119"/>
@@ -23864,7 +23895,7 @@
         <v>25</v>
       </c>
       <c r="K25" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="22.5" customHeight="1">
@@ -24162,10 +24193,10 @@
         <v>481</v>
       </c>
       <c r="B36" s="126" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="C36" s="127" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="D36" s="128"/>
       <c r="E36" s="128"/>
@@ -24181,7 +24212,7 @@
         <v>25</v>
       </c>
       <c r="K36" s="134" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="22.5" customHeight="1">
@@ -24313,7 +24344,7 @@
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="16" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="D42" s="17"/>
       <c r="E42" s="18"/>
@@ -24388,10 +24419,10 @@
         <v>484</v>
       </c>
       <c r="B46" s="107" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="C46" s="108" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="D46" s="109"/>
       <c r="E46" s="109"/>
@@ -24409,7 +24440,7 @@
         <v>74</v>
       </c>
       <c r="K46" s="115" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="22.5" customHeight="1">
@@ -24609,10 +24640,10 @@
         <v>488</v>
       </c>
       <c r="B57" s="135" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="C57" s="136" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="D57" s="137"/>
       <c r="E57" s="137"/>
@@ -24630,7 +24661,7 @@
         <v>25</v>
       </c>
       <c r="K57" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="58" spans="1:11" ht="22.5" customHeight="1">
@@ -24848,10 +24879,10 @@
         <v>491</v>
       </c>
       <c r="B68" s="107" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="C68" s="108" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="D68" s="109"/>
       <c r="E68" s="109"/>
@@ -24867,7 +24898,7 @@
         <v>74</v>
       </c>
       <c r="K68" s="115" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="69" spans="1:11" ht="22.5" customHeight="1">
@@ -25083,10 +25114,10 @@
         <v>494</v>
       </c>
       <c r="B79" s="126" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="C79" s="127" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="D79" s="128"/>
       <c r="E79" s="128"/>
@@ -25104,7 +25135,7 @@
         <v>782</v>
       </c>
       <c r="K79" s="134" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="80" spans="1:11" ht="22.5" customHeight="1">
@@ -25154,10 +25185,10 @@
         <v>497</v>
       </c>
       <c r="B82" s="117" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="C82" s="118" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="D82" s="119"/>
       <c r="E82" s="119"/>
@@ -25175,7 +25206,7 @@
         <v>74</v>
       </c>
       <c r="K82" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="83" spans="1:11" ht="22.5" customHeight="1">
@@ -25183,10 +25214,10 @@
         <v>500</v>
       </c>
       <c r="B83" s="126" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="C83" s="127" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="D83" s="128"/>
       <c r="E83" s="128"/>
@@ -25204,7 +25235,7 @@
         <v>74</v>
       </c>
       <c r="K83" s="134" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="84" spans="1:11" ht="22.5" customHeight="1">
@@ -25212,10 +25243,10 @@
         <v>451</v>
       </c>
       <c r="B84" s="151" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="C84" s="151" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="D84" s="152" t="s">
         <v>810</v>
@@ -25237,7 +25268,7 @@
         <v>25</v>
       </c>
       <c r="K84" s="158" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="85" spans="1:11" ht="22.5" customHeight="1">
@@ -25245,10 +25276,10 @@
         <v>503</v>
       </c>
       <c r="B85" s="107" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="C85" s="108" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="D85" s="109"/>
       <c r="E85" s="109"/>
@@ -25266,7 +25297,7 @@
         <v>74</v>
       </c>
       <c r="K85" s="115" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="86" spans="1:11" ht="22.5" customHeight="1">
@@ -25274,10 +25305,10 @@
         <v>506</v>
       </c>
       <c r="B86" s="135" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="C86" s="136" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="D86" s="137"/>
       <c r="E86" s="137"/>
@@ -25295,7 +25326,7 @@
         <v>74</v>
       </c>
       <c r="K86" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="87" spans="1:11" ht="22.5" customHeight="1">
@@ -25303,10 +25334,10 @@
         <v>510</v>
       </c>
       <c r="B87" s="108" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="C87" s="108" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="D87" s="109"/>
       <c r="E87" s="109"/>
@@ -25322,7 +25353,7 @@
         <v>782</v>
       </c>
       <c r="K87" s="115" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="88" spans="1:11" ht="22.5" customHeight="1">
@@ -25330,10 +25361,10 @@
         <v>514</v>
       </c>
       <c r="B88" s="135" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="C88" s="136" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="D88" s="137"/>
       <c r="E88" s="137"/>
@@ -25351,7 +25382,7 @@
         <v>74</v>
       </c>
       <c r="K88" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="89" spans="1:11" ht="22.5" customHeight="1">
@@ -25359,10 +25390,10 @@
         <v>517</v>
       </c>
       <c r="B89" s="117" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="C89" s="118" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="D89" s="70"/>
       <c r="E89" s="70"/>
@@ -25380,7 +25411,7 @@
         <v>74</v>
       </c>
       <c r="K89" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="90" spans="1:11" ht="22.5" customHeight="1">
@@ -25388,10 +25419,10 @@
         <v>520</v>
       </c>
       <c r="B90" s="135" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="C90" s="136" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="D90" s="83"/>
       <c r="E90" s="83"/>
@@ -25407,7 +25438,7 @@
         <v>74</v>
       </c>
       <c r="K90" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="91" spans="1:11" ht="22.5" customHeight="1">
@@ -25415,10 +25446,10 @@
         <v>523</v>
       </c>
       <c r="B91" s="77" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="C91" s="76" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="D91" s="70"/>
       <c r="E91" s="70"/>
@@ -25434,7 +25465,7 @@
         <v>25</v>
       </c>
       <c r="K91" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="92" spans="1:11" ht="22.5" customHeight="1">
@@ -25442,10 +25473,10 @@
         <v>527</v>
       </c>
       <c r="B92" s="81" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="C92" s="82" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="D92" s="83"/>
       <c r="E92" s="83"/>
@@ -25463,7 +25494,7 @@
         <v>74</v>
       </c>
       <c r="K92" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="93" spans="1:11" ht="22.5" customHeight="1">
@@ -25471,10 +25502,10 @@
         <v>531</v>
       </c>
       <c r="B93" s="77" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="C93" s="76" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="D93" s="70"/>
       <c r="E93" s="70"/>
@@ -25490,7 +25521,7 @@
         <v>74</v>
       </c>
       <c r="K93" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="94" spans="1:11" ht="22.5" customHeight="1">
@@ -25498,10 +25529,10 @@
         <v>534</v>
       </c>
       <c r="B94" s="81" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="C94" s="82" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="D94" s="83"/>
       <c r="E94" s="83"/>
@@ -25517,7 +25548,7 @@
         <v>74</v>
       </c>
       <c r="K94" s="143" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="95" spans="1:11" ht="22.5" customHeight="1">
@@ -25525,10 +25556,10 @@
         <v>454</v>
       </c>
       <c r="B95" s="104" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="C95" s="104" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="D95" s="62" t="s">
         <v>888</v>
@@ -25550,7 +25581,7 @@
         <v>16</v>
       </c>
       <c r="K95" s="158" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="96" spans="1:11" ht="22.5" customHeight="1">
@@ -25558,10 +25589,10 @@
         <v>538</v>
       </c>
       <c r="B96" s="77" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="C96" s="76" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="D96" s="70"/>
       <c r="E96" s="70"/>
@@ -25577,7 +25608,7 @@
         <v>74</v>
       </c>
       <c r="K96" s="125" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="97" spans="1:11" ht="22.5" customHeight="1">
@@ -25585,7 +25616,7 @@
         <v>541</v>
       </c>
       <c r="B97" s="81" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="C97" s="82" t="s">
         <v>1078</v>
@@ -25604,7 +25635,7 @@
         <v>74</v>
       </c>
       <c r="K97" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="98" spans="1:11" ht="22.5" customHeight="1">
@@ -25612,10 +25643,10 @@
         <v>544</v>
       </c>
       <c r="B98" s="77" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="C98" s="76" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="D98" s="70"/>
       <c r="E98" s="70"/>
@@ -25633,7 +25664,7 @@
         <v>74</v>
       </c>
       <c r="K98" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="99" spans="1:11" ht="22.5" customHeight="1">
@@ -25641,10 +25672,10 @@
         <v>547</v>
       </c>
       <c r="B99" s="81" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="C99" s="82" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="D99" s="83"/>
       <c r="E99" s="83"/>
@@ -25662,7 +25693,7 @@
         <v>74</v>
       </c>
       <c r="K99" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="100" spans="1:11" ht="22.5" customHeight="1">
@@ -25670,10 +25701,10 @@
         <v>552</v>
       </c>
       <c r="B100" s="77" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="C100" s="76" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="D100" s="70"/>
       <c r="E100" s="70"/>
@@ -25689,7 +25720,7 @@
         <v>74</v>
       </c>
       <c r="K100" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="101" spans="1:11" ht="22.5" customHeight="1">
@@ -25697,10 +25728,10 @@
         <v>555</v>
       </c>
       <c r="B101" s="81" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="C101" s="82" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="D101" s="83"/>
       <c r="E101" s="83"/>
@@ -25716,7 +25747,7 @@
         <v>74</v>
       </c>
       <c r="K101" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="102" spans="1:11" ht="22.5" customHeight="1">
@@ -25724,10 +25755,10 @@
         <v>558</v>
       </c>
       <c r="B102" s="77" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="C102" s="76" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="D102" s="70"/>
       <c r="E102" s="70"/>
@@ -25743,7 +25774,7 @@
         <v>74</v>
       </c>
       <c r="K102" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="103" spans="1:11" ht="22.5" customHeight="1">
@@ -25751,10 +25782,10 @@
         <v>562</v>
       </c>
       <c r="B103" s="81" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="C103" s="82" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="D103" s="83"/>
       <c r="E103" s="83"/>
@@ -25770,7 +25801,7 @@
         <v>74</v>
       </c>
       <c r="K103" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="104" spans="1:11" ht="22.5" customHeight="1">
@@ -25778,10 +25809,10 @@
         <v>565</v>
       </c>
       <c r="B104" s="76" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="C104" s="76" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="D104" s="70"/>
       <c r="E104" s="70"/>
@@ -25799,7 +25830,7 @@
         <v>25</v>
       </c>
       <c r="K104" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="105" spans="1:11" ht="22.5" customHeight="1">
@@ -25807,10 +25838,10 @@
         <v>568</v>
       </c>
       <c r="B105" s="81" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="C105" s="82" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="D105" s="83"/>
       <c r="E105" s="83"/>
@@ -25828,7 +25859,7 @@
         <v>74</v>
       </c>
       <c r="K105" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="106" spans="1:11" ht="22.5" customHeight="1">
@@ -25836,10 +25867,10 @@
         <v>457</v>
       </c>
       <c r="B106" s="104" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="C106" s="104" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="D106" s="62" t="s">
         <v>540</v>
@@ -25861,7 +25892,7 @@
         <v>1192</v>
       </c>
       <c r="K106" s="104" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="107" spans="1:11" ht="22.5" customHeight="1">
@@ -25869,10 +25900,10 @@
         <v>571</v>
       </c>
       <c r="B107" s="77" t="s">
-        <v>1372</v>
+        <v>1373</v>
       </c>
       <c r="C107" s="76" t="s">
-        <v>1373</v>
+        <v>1374</v>
       </c>
       <c r="D107" s="70"/>
       <c r="E107" s="70"/>
@@ -25888,7 +25919,7 @@
         <v>25</v>
       </c>
       <c r="K107" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="108" spans="1:11" ht="22.5" customHeight="1">
@@ -25896,10 +25927,10 @@
         <v>574</v>
       </c>
       <c r="B108" s="81" t="s">
-        <v>1374</v>
+        <v>1375</v>
       </c>
       <c r="C108" s="82" t="s">
-        <v>1375</v>
+        <v>1376</v>
       </c>
       <c r="D108" s="83"/>
       <c r="E108" s="83"/>
@@ -25915,7 +25946,7 @@
         <v>74</v>
       </c>
       <c r="K108" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="109" spans="1:11" ht="22.5" customHeight="1">
@@ -25923,10 +25954,10 @@
         <v>576</v>
       </c>
       <c r="B109" s="77" t="s">
-        <v>1376</v>
+        <v>1377</v>
       </c>
       <c r="C109" s="76" t="s">
-        <v>1377</v>
+        <v>1378</v>
       </c>
       <c r="D109" s="70"/>
       <c r="E109" s="70"/>
@@ -25944,7 +25975,7 @@
         <v>25</v>
       </c>
       <c r="K109" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="110" spans="1:11" ht="22.5" customHeight="1">
@@ -25952,10 +25983,10 @@
         <v>579</v>
       </c>
       <c r="B110" s="81" t="s">
-        <v>1378</v>
+        <v>1379</v>
       </c>
       <c r="C110" s="82" t="s">
-        <v>1379</v>
+        <v>1380</v>
       </c>
       <c r="D110" s="83"/>
       <c r="E110" s="83"/>
@@ -25971,7 +26002,7 @@
         <v>74</v>
       </c>
       <c r="K110" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="111" spans="1:11" ht="22.5" customHeight="1">
@@ -25979,10 +26010,10 @@
         <v>582</v>
       </c>
       <c r="B111" s="77" t="s">
-        <v>1380</v>
+        <v>1381</v>
       </c>
       <c r="C111" s="76" t="s">
-        <v>1381</v>
+        <v>1382</v>
       </c>
       <c r="D111" s="70"/>
       <c r="E111" s="70"/>
@@ -25998,7 +26029,7 @@
         <v>74</v>
       </c>
       <c r="K111" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="112" spans="1:11" ht="22.5" customHeight="1">
@@ -26006,10 +26037,10 @@
         <v>585</v>
       </c>
       <c r="B112" s="81" t="s">
-        <v>1382</v>
+        <v>1383</v>
       </c>
       <c r="C112" s="82" t="s">
-        <v>1383</v>
+        <v>1384</v>
       </c>
       <c r="D112" s="83"/>
       <c r="E112" s="83"/>
@@ -26025,7 +26056,7 @@
         <v>74</v>
       </c>
       <c r="K112" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="113" spans="1:11" ht="22.5" customHeight="1">
@@ -26033,10 +26064,10 @@
         <v>588</v>
       </c>
       <c r="B113" s="77" t="s">
-        <v>1384</v>
+        <v>1385</v>
       </c>
       <c r="C113" s="76" t="s">
-        <v>1385</v>
+        <v>1386</v>
       </c>
       <c r="D113" s="70"/>
       <c r="E113" s="70"/>
@@ -26052,7 +26083,7 @@
         <v>74</v>
       </c>
       <c r="K113" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="114" spans="1:11" ht="22.5" customHeight="1">
@@ -26060,10 +26091,10 @@
         <v>591</v>
       </c>
       <c r="B114" s="81" t="s">
-        <v>1386</v>
+        <v>1387</v>
       </c>
       <c r="C114" s="82" t="s">
-        <v>1387</v>
+        <v>1388</v>
       </c>
       <c r="D114" s="83"/>
       <c r="E114" s="83"/>
@@ -26079,7 +26110,7 @@
         <v>74</v>
       </c>
       <c r="K114" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="115" spans="1:11" ht="22.5" customHeight="1">
@@ -26087,7 +26118,7 @@
         <v>594</v>
       </c>
       <c r="B115" s="77" t="s">
-        <v>1388</v>
+        <v>1389</v>
       </c>
       <c r="C115" s="76" t="s">
         <v>391</v>
@@ -26106,7 +26137,7 @@
         <v>74</v>
       </c>
       <c r="K115" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="116" spans="1:11" ht="22.5" customHeight="1">
@@ -26114,10 +26145,10 @@
         <v>597</v>
       </c>
       <c r="B116" s="81" t="s">
-        <v>1389</v>
+        <v>1390</v>
       </c>
       <c r="C116" s="82" t="s">
-        <v>1390</v>
+        <v>1391</v>
       </c>
       <c r="D116" s="83"/>
       <c r="E116" s="83"/>
@@ -26133,7 +26164,7 @@
         <v>74</v>
       </c>
       <c r="K116" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="117" spans="1:11" ht="22.5" customHeight="1">
@@ -26141,10 +26172,10 @@
         <v>668</v>
       </c>
       <c r="B117" s="104" t="s">
-        <v>1391</v>
+        <v>1392</v>
       </c>
       <c r="C117" s="104" t="s">
-        <v>1392</v>
+        <v>1393</v>
       </c>
       <c r="D117" s="62" t="s">
         <v>540</v>
@@ -26166,7 +26197,7 @@
         <v>1192</v>
       </c>
       <c r="K117" s="104" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="118" spans="1:11" ht="22.5" customHeight="1">
@@ -26174,10 +26205,10 @@
         <v>600</v>
       </c>
       <c r="B118" s="77" t="s">
-        <v>1393</v>
+        <v>1394</v>
       </c>
       <c r="C118" s="76" t="s">
-        <v>1394</v>
+        <v>1395</v>
       </c>
       <c r="D118" s="70"/>
       <c r="E118" s="70"/>
@@ -26193,7 +26224,7 @@
         <v>74</v>
       </c>
       <c r="K118" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="119" spans="1:11" ht="22.5" customHeight="1">
@@ -26201,10 +26232,10 @@
         <v>603</v>
       </c>
       <c r="B119" s="81" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="C119" s="82" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="D119" s="83"/>
       <c r="E119" s="83"/>
@@ -26222,7 +26253,7 @@
         <v>74</v>
       </c>
       <c r="K119" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="120" spans="1:11" ht="22.5" customHeight="1">
@@ -26230,10 +26261,10 @@
         <v>606</v>
       </c>
       <c r="B120" s="77" t="s">
-        <v>1395</v>
+        <v>1396</v>
       </c>
       <c r="C120" s="76" t="s">
-        <v>1396</v>
+        <v>1397</v>
       </c>
       <c r="D120" s="70"/>
       <c r="E120" s="70"/>
@@ -26251,7 +26282,7 @@
         <v>74</v>
       </c>
       <c r="K120" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="121" spans="1:11" ht="22.5" customHeight="1">
@@ -26259,10 +26290,10 @@
         <v>609</v>
       </c>
       <c r="B121" s="81" t="s">
-        <v>1397</v>
+        <v>1398</v>
       </c>
       <c r="C121" s="82" t="s">
-        <v>1398</v>
+        <v>1399</v>
       </c>
       <c r="D121" s="83"/>
       <c r="E121" s="83"/>
@@ -26278,7 +26309,7 @@
         <v>74</v>
       </c>
       <c r="K121" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="122" spans="1:11" ht="22.5" customHeight="1">
@@ -26286,10 +26317,10 @@
         <v>612</v>
       </c>
       <c r="B122" s="77" t="s">
-        <v>1399</v>
+        <v>1400</v>
       </c>
       <c r="C122" s="76" t="s">
-        <v>1400</v>
+        <v>1401</v>
       </c>
       <c r="D122" s="70"/>
       <c r="E122" s="70"/>
@@ -26305,7 +26336,7 @@
         <v>74</v>
       </c>
       <c r="K122" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="123" spans="1:11" ht="22.5" customHeight="1">
@@ -26313,10 +26344,10 @@
         <v>615</v>
       </c>
       <c r="B123" s="81" t="s">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="C123" s="82" t="s">
-        <v>1402</v>
+        <v>1403</v>
       </c>
       <c r="D123" s="83"/>
       <c r="E123" s="83"/>
@@ -26332,7 +26363,7 @@
         <v>74</v>
       </c>
       <c r="K123" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="124" spans="1:11" ht="22.5" customHeight="1">
@@ -26340,10 +26371,10 @@
         <v>618</v>
       </c>
       <c r="B124" s="77" t="s">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="C124" s="76" t="s">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="D124" s="70"/>
       <c r="E124" s="70"/>
@@ -26361,7 +26392,7 @@
         <v>25</v>
       </c>
       <c r="K124" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="125" spans="1:11" ht="22.5" customHeight="1">
@@ -26369,10 +26400,10 @@
         <v>621</v>
       </c>
       <c r="B125" s="81" t="s">
-        <v>1405</v>
+        <v>1406</v>
       </c>
       <c r="C125" s="82" t="s">
-        <v>1406</v>
+        <v>1407</v>
       </c>
       <c r="D125" s="83"/>
       <c r="E125" s="83"/>
@@ -26388,7 +26419,7 @@
         <v>25</v>
       </c>
       <c r="K125" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="126" spans="1:11" ht="22.5" customHeight="1">
@@ -26396,10 +26427,10 @@
         <v>624</v>
       </c>
       <c r="B126" s="77" t="s">
-        <v>1407</v>
+        <v>1408</v>
       </c>
       <c r="C126" s="76" t="s">
-        <v>1408</v>
+        <v>1409</v>
       </c>
       <c r="D126" s="70"/>
       <c r="E126" s="70"/>
@@ -26415,7 +26446,7 @@
         <v>74</v>
       </c>
       <c r="K126" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="127" spans="1:11" ht="22.5" customHeight="1">
@@ -26423,10 +26454,10 @@
         <v>627</v>
       </c>
       <c r="B127" s="81" t="s">
-        <v>1409</v>
+        <v>1410</v>
       </c>
       <c r="C127" s="82" t="s">
-        <v>1410</v>
+        <v>1411</v>
       </c>
       <c r="D127" s="83"/>
       <c r="E127" s="83"/>
@@ -26442,7 +26473,7 @@
         <v>74</v>
       </c>
       <c r="K127" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="128" spans="1:11" ht="22.5" customHeight="1">
@@ -26450,10 +26481,10 @@
         <v>459</v>
       </c>
       <c r="B128" s="104" t="s">
-        <v>1411</v>
+        <v>1412</v>
       </c>
       <c r="C128" s="104" t="s">
-        <v>1412</v>
+        <v>1413</v>
       </c>
       <c r="D128" s="62" t="s">
         <v>540</v>
@@ -26475,7 +26506,7 @@
         <v>1036</v>
       </c>
       <c r="K128" s="104" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="22.5" customHeight="1">
@@ -26483,10 +26514,10 @@
         <v>630</v>
       </c>
       <c r="B129" s="77" t="s">
-        <v>1413</v>
+        <v>1414</v>
       </c>
       <c r="C129" s="76" t="s">
-        <v>1414</v>
+        <v>1415</v>
       </c>
       <c r="D129" s="70"/>
       <c r="E129" s="70"/>
@@ -26502,7 +26533,7 @@
         <v>74</v>
       </c>
       <c r="K129" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="22.5" customHeight="1">
@@ -26510,10 +26541,10 @@
         <v>633</v>
       </c>
       <c r="B130" s="81" t="s">
-        <v>1415</v>
+        <v>1416</v>
       </c>
       <c r="C130" s="82" t="s">
-        <v>1416</v>
+        <v>1417</v>
       </c>
       <c r="D130" s="83"/>
       <c r="E130" s="83"/>
@@ -26531,7 +26562,7 @@
         <v>74</v>
       </c>
       <c r="K130" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="131" spans="1:11" ht="22.5" customHeight="1">
@@ -26539,10 +26570,10 @@
         <v>636</v>
       </c>
       <c r="B131" s="77" t="s">
-        <v>1417</v>
+        <v>1418</v>
       </c>
       <c r="C131" s="76" t="s">
-        <v>1418</v>
+        <v>1419</v>
       </c>
       <c r="D131" s="70"/>
       <c r="E131" s="70"/>
@@ -26558,7 +26589,7 @@
         <v>74</v>
       </c>
       <c r="K131" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="132" spans="1:11" ht="22.5" customHeight="1">
@@ -26566,10 +26597,10 @@
         <v>637</v>
       </c>
       <c r="B132" s="81" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="C132" s="82" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="D132" s="83"/>
       <c r="E132" s="83"/>
@@ -26587,7 +26618,7 @@
         <v>74</v>
       </c>
       <c r="K132" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="133" spans="1:11" ht="22.5" customHeight="1">
@@ -26595,10 +26626,10 @@
         <v>638</v>
       </c>
       <c r="B133" s="77" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="C133" s="76" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="D133" s="70"/>
       <c r="E133" s="70"/>
@@ -26616,7 +26647,7 @@
         <v>25</v>
       </c>
       <c r="K133" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="134" spans="1:11" ht="22.5" customHeight="1">
@@ -26624,10 +26655,10 @@
         <v>639</v>
       </c>
       <c r="B134" s="81" t="s">
-        <v>1419</v>
+        <v>1420</v>
       </c>
       <c r="C134" s="82" t="s">
-        <v>1420</v>
+        <v>1421</v>
       </c>
       <c r="D134" s="83"/>
       <c r="E134" s="83"/>
@@ -26643,7 +26674,7 @@
         <v>25</v>
       </c>
       <c r="K134" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="135" spans="1:11" ht="22.5" customHeight="1">
@@ -26651,10 +26682,10 @@
         <v>640</v>
       </c>
       <c r="B135" s="77" t="s">
-        <v>1421</v>
+        <v>1422</v>
       </c>
       <c r="C135" s="76" t="s">
-        <v>1422</v>
+        <v>1423</v>
       </c>
       <c r="D135" s="70"/>
       <c r="E135" s="70"/>
@@ -26672,7 +26703,7 @@
         <v>25</v>
       </c>
       <c r="K135" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="136" spans="1:11" ht="22.5" customHeight="1">
@@ -26680,10 +26711,10 @@
         <v>641</v>
       </c>
       <c r="B136" s="81" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="C136" s="82" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="D136" s="83"/>
       <c r="E136" s="83"/>
@@ -26699,7 +26730,7 @@
         <v>74</v>
       </c>
       <c r="K136" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="137" spans="1:11" ht="22.5" customHeight="1">
@@ -26707,10 +26738,10 @@
         <v>642</v>
       </c>
       <c r="B137" s="77" t="s">
-        <v>1423</v>
+        <v>1424</v>
       </c>
       <c r="C137" s="76" t="s">
-        <v>1424</v>
+        <v>1425</v>
       </c>
       <c r="D137" s="70"/>
       <c r="E137" s="70"/>
@@ -26726,7 +26757,7 @@
         <v>74</v>
       </c>
       <c r="K137" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="138" spans="1:11" ht="22.5" customHeight="1">
@@ -26734,10 +26765,10 @@
         <v>643</v>
       </c>
       <c r="B138" s="81" t="s">
-        <v>1425</v>
+        <v>1426</v>
       </c>
       <c r="C138" s="82" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="D138" s="83"/>
       <c r="E138" s="83"/>
@@ -26755,7 +26786,7 @@
         <v>74</v>
       </c>
       <c r="K138" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="139" spans="1:11" ht="22.5" customHeight="1">
@@ -26763,10 +26794,10 @@
         <v>462</v>
       </c>
       <c r="B139" s="104" t="s">
-        <v>1426</v>
+        <v>1427</v>
       </c>
       <c r="C139" s="104" t="s">
-        <v>1427</v>
+        <v>1428</v>
       </c>
       <c r="D139" s="62" t="s">
         <v>810</v>
@@ -26788,7 +26819,7 @@
         <v>25</v>
       </c>
       <c r="K139" s="104" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="140" spans="1:11" ht="22.5" customHeight="1">
@@ -26796,10 +26827,10 @@
         <v>644</v>
       </c>
       <c r="B140" s="81" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="C140" s="82" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
       <c r="D140" s="83"/>
       <c r="E140" s="83"/>
@@ -26817,7 +26848,7 @@
         <v>74</v>
       </c>
       <c r="K140" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="141" spans="1:11" ht="22.5" customHeight="1">
@@ -26825,10 +26856,10 @@
         <v>645</v>
       </c>
       <c r="B141" s="77" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="C141" s="76" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="D141" s="70"/>
       <c r="E141" s="70"/>
@@ -26844,7 +26875,7 @@
         <v>25</v>
       </c>
       <c r="K141" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="142" spans="1:11" ht="22.5" customHeight="1">
@@ -26852,7 +26883,7 @@
         <v>646</v>
       </c>
       <c r="B142" s="81" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="C142" s="82" t="s">
         <v>1094</v>
@@ -26871,7 +26902,7 @@
         <v>74</v>
       </c>
       <c r="K142" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="143" spans="1:11" ht="22.5" customHeight="1">
@@ -26879,10 +26910,10 @@
         <v>647</v>
       </c>
       <c r="B143" s="77" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="C143" s="76" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="D143" s="70"/>
       <c r="E143" s="70"/>
@@ -26898,7 +26929,7 @@
         <v>74</v>
       </c>
       <c r="K143" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="144" spans="1:11" ht="22.5" customHeight="1">
@@ -26906,10 +26937,10 @@
         <v>648</v>
       </c>
       <c r="B144" s="81" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
       <c r="C144" s="82" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="D144" s="83"/>
       <c r="E144" s="83"/>
@@ -26925,7 +26956,7 @@
         <v>74</v>
       </c>
       <c r="K144" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="145" spans="1:11" ht="22.5" customHeight="1">
@@ -26933,10 +26964,10 @@
         <v>649</v>
       </c>
       <c r="B145" s="77" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="C145" s="76" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="D145" s="70"/>
       <c r="E145" s="70"/>
@@ -26952,7 +26983,7 @@
         <v>25</v>
       </c>
       <c r="K145" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="146" spans="1:11" ht="22.5" customHeight="1">
@@ -26960,10 +26991,10 @@
         <v>650</v>
       </c>
       <c r="B146" s="81" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
       <c r="C146" s="82" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="D146" s="83"/>
       <c r="E146" s="83"/>
@@ -26979,7 +27010,7 @@
         <v>74</v>
       </c>
       <c r="K146" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="147" spans="1:11" ht="22.5" customHeight="1">
@@ -26987,10 +27018,10 @@
         <v>651</v>
       </c>
       <c r="B147" s="77" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="C147" s="76" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="D147" s="70"/>
       <c r="E147" s="70"/>
@@ -27006,7 +27037,7 @@
         <v>25</v>
       </c>
       <c r="K147" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="148" spans="1:11" ht="22.5" customHeight="1">
@@ -27014,10 +27045,10 @@
         <v>652</v>
       </c>
       <c r="B148" s="81" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="C148" s="82" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="D148" s="83"/>
       <c r="E148" s="83"/>
@@ -27033,7 +27064,7 @@
         <v>74</v>
       </c>
       <c r="K148" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="149" spans="1:11" ht="22.5" customHeight="1">
@@ -27041,10 +27072,10 @@
         <v>653</v>
       </c>
       <c r="B149" s="77" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="C149" s="76" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="D149" s="70"/>
       <c r="E149" s="70"/>
@@ -27060,7 +27091,7 @@
         <v>74</v>
       </c>
       <c r="K149" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="150" spans="1:11" ht="22.5" customHeight="1">
@@ -27068,7 +27099,7 @@
         <v>465</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="C150" s="2"/>
       <c r="D150" s="166" t="s">
@@ -27087,10 +27118,10 @@
         <v>654</v>
       </c>
       <c r="B151" s="82" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="C151" s="82" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="D151" s="83"/>
       <c r="E151" s="83"/>
@@ -27106,7 +27137,7 @@
         <v>782</v>
       </c>
       <c r="K151" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="152" spans="1:11" ht="22.5" customHeight="1">
@@ -27114,10 +27145,10 @@
         <v>746</v>
       </c>
       <c r="B152" s="77" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="C152" s="76" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="D152" s="70"/>
       <c r="E152" s="70"/>
@@ -27133,7 +27164,7 @@
         <v>25</v>
       </c>
       <c r="K152" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="153" spans="1:11" ht="22.5" customHeight="1">
@@ -27141,10 +27172,10 @@
         <v>747</v>
       </c>
       <c r="B153" s="81" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="C153" s="82" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="D153" s="83"/>
       <c r="E153" s="83"/>
@@ -27160,7 +27191,7 @@
         <v>74</v>
       </c>
       <c r="K153" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="154" spans="1:11" ht="22.5" customHeight="1">
@@ -27168,10 +27199,10 @@
         <v>748</v>
       </c>
       <c r="B154" s="77" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="C154" s="76" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="D154" s="70"/>
       <c r="E154" s="70"/>
@@ -27187,7 +27218,7 @@
         <v>25</v>
       </c>
       <c r="K154" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="155" spans="1:11" ht="22.5" customHeight="1">
@@ -27195,10 +27226,10 @@
         <v>749</v>
       </c>
       <c r="B155" s="81" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="C155" s="82" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="D155" s="83"/>
       <c r="E155" s="83"/>
@@ -27216,7 +27247,7 @@
         <v>25</v>
       </c>
       <c r="K155" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="156" spans="1:11" ht="22.5" customHeight="1">
@@ -27224,10 +27255,10 @@
         <v>750</v>
       </c>
       <c r="B156" s="76" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="C156" s="76" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="D156" s="70"/>
       <c r="E156" s="70"/>
@@ -27243,7 +27274,7 @@
         <v>513</v>
       </c>
       <c r="K156" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="157" spans="1:11" ht="22.5" customHeight="1">
@@ -27251,10 +27282,10 @@
         <v>751</v>
       </c>
       <c r="B157" s="81" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="C157" s="82" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="D157" s="83"/>
       <c r="E157" s="83"/>
@@ -27272,7 +27303,7 @@
         <v>74</v>
       </c>
       <c r="K157" s="82" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="158" spans="1:11" ht="22.5" customHeight="1">
@@ -27280,10 +27311,10 @@
         <v>752</v>
       </c>
       <c r="B158" s="76" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="C158" s="76" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="D158" s="70"/>
       <c r="E158" s="70"/>
@@ -27301,7 +27332,7 @@
         <v>25</v>
       </c>
       <c r="K158" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="159" spans="1:11" ht="22.5" customHeight="1">
@@ -27309,10 +27340,10 @@
         <v>753</v>
       </c>
       <c r="B159" s="77" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
       <c r="C159" s="76" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
       <c r="D159" s="10"/>
       <c r="E159" s="11"/>
@@ -27328,7 +27359,7 @@
         <v>25</v>
       </c>
       <c r="K159" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="160" spans="1:11" ht="22.5" customHeight="1">
@@ -27336,10 +27367,10 @@
         <v>754</v>
       </c>
       <c r="B160" s="77" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
       <c r="C160" s="76" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="D160" s="10"/>
       <c r="E160" s="11"/>
@@ -27355,7 +27386,7 @@
         <v>25</v>
       </c>
       <c r="K160" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="161" spans="1:11" ht="22.5" customHeight="1">
@@ -27380,10 +27411,10 @@
         <v>755</v>
       </c>
       <c r="B162" s="9" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="C162" s="9" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
       <c r="D162" s="10"/>
       <c r="E162" s="11"/>
@@ -27401,7 +27432,7 @@
         <v>74</v>
       </c>
       <c r="K162" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="163" spans="1:11" ht="22.5" customHeight="1">
@@ -27409,10 +27440,10 @@
         <v>756</v>
       </c>
       <c r="B163" s="9" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="C163" s="9" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="D163" s="10"/>
       <c r="E163" s="11"/>
@@ -27430,7 +27461,7 @@
         <v>25</v>
       </c>
       <c r="K163" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="164" spans="1:11" ht="22.5" customHeight="1">
@@ -27438,10 +27469,10 @@
         <v>757</v>
       </c>
       <c r="B164" s="9" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="C164" s="9" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="D164" s="10"/>
       <c r="E164" s="11"/>
@@ -27459,7 +27490,7 @@
         <v>745</v>
       </c>
       <c r="K164" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="165" spans="1:11" ht="22.5" customHeight="1">
@@ -27467,10 +27498,10 @@
         <v>758</v>
       </c>
       <c r="B165" s="9" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="C165" s="9" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="D165" s="10"/>
       <c r="E165" s="11"/>
@@ -27488,7 +27519,7 @@
         <v>551</v>
       </c>
       <c r="K165" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="166" spans="1:11" ht="22.5" customHeight="1">
@@ -27525,10 +27556,10 @@
         <v>11</v>
       </c>
       <c r="B167" s="9" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="C167" s="9" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="D167" s="10"/>
       <c r="E167" s="11"/>
@@ -27546,7 +27577,7 @@
         <v>551</v>
       </c>
       <c r="K167" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="168" spans="1:11" ht="22.5" customHeight="1">
@@ -27583,10 +27614,10 @@
         <v>18</v>
       </c>
       <c r="B169" s="9" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C169" s="9" t="s">
         <v>1271</v>
-      </c>
-      <c r="C169" s="9" t="s">
-        <v>1270</v>
       </c>
       <c r="D169" s="10"/>
       <c r="E169" s="11"/>
@@ -27604,7 +27635,7 @@
         <v>551</v>
       </c>
       <c r="K169" s="76" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="170" spans="1:11" ht="22.5" customHeight="1">
@@ -29156,10 +29187,10 @@
     <row r="248" spans="1:11" ht="22.5" customHeight="1">
       <c r="A248" s="46"/>
       <c r="B248" s="9" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="C248" s="9" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
       <c r="D248" s="10"/>
       <c r="E248" s="48" t="s">

</xml_diff>